<commit_message>
Reinstate _reviewPRNsAndPERNs resx's from main and re-add resources; Rengenerated translations
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/multi-year/xlsx/06-obligations-home-no-obligations.xlsx
+++ b/translations/welsh-translations/multi-year/xlsx/06-obligations-home-no-obligations.xlsx
@@ -276,7 +276,7 @@
     <row r="9" ht="51" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::review_your_prns_and_perns_year</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_reviewPRNsAndPERNs.en.resx::review_your_prns_and_perns_yyyy</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -286,7 +286,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">review_your_prns_and_perns_year</t>
+          <t xml:space="preserve">review_your_prns_and_perns_yyyy</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">

</xml_diff>